<commit_message>
docs(adsense): track consent implementation and editorial gaps
</commit_message>
<xml_diff>
--- a/outputs/project-tracker-2026-09-27-adsense/Comparador-Hardware-Project-Tracker.xlsx
+++ b/outputs/project-tracker-2026-09-27-adsense/Comparador-Hardware-Project-Tracker.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Plan" sheetId="1" r:id="Ra5a7e6e9e1614ef2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Plan" sheetId="1" r:id="R9202dd6906a94c60"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -612,7 +612,7 @@
         <x:color rgb="FF087E5D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDDF8F3"/>
         </x:patternFill>
       </x:fill>
@@ -623,7 +623,7 @@
         <x:color rgb="FF3258CD"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE7EEFF"/>
         </x:patternFill>
       </x:fill>
@@ -634,7 +634,7 @@
         <x:color rgb="FFC23647"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE3EA"/>
         </x:patternFill>
       </x:fill>
@@ -644,7 +644,7 @@
         <x:color rgb="FF7745C3"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF1E9FF"/>
         </x:patternFill>
       </x:fill>
@@ -655,7 +655,7 @@
         <x:color rgb="FFC23647"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE3EA"/>
         </x:patternFill>
       </x:fill>
@@ -666,7 +666,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -677,35 +677,35 @@
         <x:color rgb="FF7745C3"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF1E9FF"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FF00BFA6"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FF4D7CFE"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFF6675"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFA977F6"/>
         </x:patternFill>
       </x:fill>
@@ -1254,7 +1254,7 @@
       <x:c r="R6" s="47"/>
       <x:c r="S6" s="35" t="n">
         <x:f>COUNTIF($E$10:$E$49,"In Progress")</x:f>
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="T6" s="36"/>
       <x:c r="U6" s="36"/>
@@ -4609,27 +4609,28 @@
         <x:v>Jonathan + Codex</x:v>
       </x:c>
       <x:c r="E44" s="66" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="F44" s="66" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="G44" s="68" t="n">
-        <x:v>46296.5</x:v>
+        <x:v>46292.5</x:v>
       </x:c>
       <x:c r="H44" s="68" t="n">
         <x:v>46302.5</x:v>
       </x:c>
       <x:c r="I44" s="69" t="n">
         <x:f>IF(OR(G44="",H44="",H44&lt;G44),"",H44-G44+1)</x:f>
-        <x:v>7</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="J44"/>
       <x:c r="K44" s="70" t="str">
         <x:f>IF(OR($G44="",$H44="",$H44&lt;$G44),"",IF(AND(K$9&lt;=$H44,K$9+6&gt;=$G44),1,""))</x:f>
       </x:c>
-      <x:c r="L44" s="70" t="str">
+      <x:c r="L44" s="70" t="n">
         <x:f>IF(OR($G44="",$H44="",$H44&lt;$G44),"",IF(AND(L$9&lt;=$H44,L$9+6&gt;=$G44),1,""))</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M44" s="70" t="n">
         <x:f>IF(OR($G44="",$H44="",$H44&lt;$G44),"",IF(AND(M$9&lt;=$H44,M$9+6&gt;=$G44),1,""))</x:f>
@@ -5140,7 +5141,7 @@
     </x:row>
     <x:row r="50" ht="72" customHeight="1">
       <x:c r="B50" s="61" t="str">
-        <x:v>Fuentes: REVISION-Y-PLAN.md; BACKLOG.csv; METRICAS.csv; VALIDACION.md; Search Console y GA4 consultados el 21/09/2026. GSC 23/08–19/09 vs 26/07–22/08: 296 vs 192 clics, 14 mil vs 9,55 mil impresiones, CTR 2,1% vs 2,0%, posición 8,4 vs 8,5. Auditoría GSC: 3.187 indexadas / 326 no indexadas; sitemap correcto con 29 páginas descubiertas; HTTPS 31/0; 2 enlaces externos y 7.751 internos; 662 oportunidades Merchant; sin acciones manuales ni problemas de seguridad; sin datos CrUX. GA4 24/08–20/09: 143 usuarios, 512 eventos, 178 page_view y 18 click; generate_lead aún no aparece. Jev 21/09: embudo/CTA 64% (confianza 0,56); enlaces/rich results 39% y asociación GA4 32% como segundo orden (confianza 0,23); Merchant 6% y outreach 26% a favor. G07 pasa a P0/en curso; G17 a P1. Las fechas futuras son planificación y se revisan semanalmente. G02 25/09: 64/47.727 ofertas disponibles con observación ≤24 h antes del ciclo medido; 80 observaciones persistidas en 11 tiendas en run 36164068314; despacho automático verificado en runs 36165637147 y 36166218562. G02 sigue en observación; próxima revisión tras siete ciclos útiles medidos el 03/10. Fuente: VALIDACION.md y FRESCURA-TIENDAS-2026-09-25.csv. Actualización 27/09/2026: PLAN-ADSENSE-2026-09-27.md y BACKLOG.csv G18–G26. Fechas propuestas y dependientes de cuenta, contenido, privacidad y aprobación externa; anuncios no activos. Cuenta existente confirmada por Jonathan; país y método de cobro requieren comprobación. Fuente de políticas: https://support.google.com/adsense/answer/9724?hl=es. QVL y difusión conservan sus cortes históricos.</x:v>
+        <x:v>Fuentes: REVISION-Y-PLAN.md; BACKLOG.csv; METRICAS.csv; VALIDACION.md; Search Console y GA4 consultados el 21/09/2026. GSC 23/08–19/09 vs 26/07–22/08: 296 vs 192 clics, 14 mil vs 9,55 mil impresiones, CTR 2,1% vs 2,0%, posición 8,4 vs 8,5. Auditoría GSC: 3.187 indexadas / 326 no indexadas; sitemap correcto con 29 páginas descubiertas; HTTPS 31/0; 2 enlaces externos y 7.751 internos; 662 oportunidades Merchant; sin acciones manuales ni problemas de seguridad; sin datos CrUX. GA4 24/08–20/09: 143 usuarios, 512 eventos, 178 page_view y 18 click; generate_lead aún no aparece. Jev 21/09: embudo/CTA 64% (confianza 0,56); enlaces/rich results 39% y asociación GA4 32% como segundo orden (confianza 0,23); Merchant 6% y outreach 26% a favor. G07 pasa a P0/en curso; G17 a P1. Las fechas futuras son planificación y se revisan semanalmente. G02 25/09: 64/47.727 ofertas disponibles con observación ≤24 h antes del ciclo medido; 80 observaciones persistidas en 11 tiendas en run 36164068314; despacho automático verificado en runs 36165637147 y 36166218562. G02 sigue en observación; próxima revisión tras siete ciclos útiles medidos el 03/10. Fuente: VALIDACION.md y FRESCURA-TIENDAS-2026-09-25.csv. Actualización 27/09/2026: PLAN-ADSENSE-2026-09-27.md y BACKLOG.csv G18–G26. Fechas propuestas y dependientes de cuenta, contenido, privacidad y aprobación externa; anuncios no activos. Cuenta existente confirmada por Jonathan; país y método de cobro requieren comprobación. Fuente de políticas: https://support.google.com/adsense/answer/9724?hl=es. QVL y difusión conservan sus cortes históricos. Corte 27/09: G21 iniciado, consentimiento GA4 básico y política implementados; 19 pruebas y navegador local desktop/móvil verificados. Publicación, recepción del contacto y CMP de anuncios pendientes. G19 mantiene revisión y registro de derechos pendiente. No aprobado para AdSense.</x:v>
       </x:c>
       <x:c r="C50" s="61"/>
       <x:c r="D50" s="61"/>

</xml_diff>

<commit_message>
docs(adsense): record editorial preparation and payment prerequisites
</commit_message>
<xml_diff>
--- a/outputs/project-tracker-2026-09-27-adsense/Comparador-Hardware-Project-Tracker.xlsx
+++ b/outputs/project-tracker-2026-09-27-adsense/Comparador-Hardware-Project-Tracker.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Plan" sheetId="1" r:id="R9202dd6906a94c60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Plan" sheetId="1" r:id="R38f1cadb5da44abf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1254,7 +1254,7 @@
       <x:c r="R6" s="47"/>
       <x:c r="S6" s="35" t="n">
         <x:f>COUNTIF($E$10:$E$49,"In Progress")</x:f>
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="T6" s="36"/>
       <x:c r="U6" s="36"/>
@@ -4519,27 +4519,28 @@
         <x:v>Jonathan + Codex</x:v>
       </x:c>
       <x:c r="E43" s="66" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="F43" s="66" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="G43" s="68" t="n">
-        <x:v>46296.5</x:v>
+        <x:v>46292.5</x:v>
       </x:c>
       <x:c r="H43" s="68" t="n">
         <x:v>46302.5</x:v>
       </x:c>
       <x:c r="I43" s="69" t="n">
         <x:f>IF(OR(G43="",H43="",H43&lt;G43),"",H43-G43+1)</x:f>
-        <x:v>7</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="J43"/>
       <x:c r="K43" s="70" t="str">
         <x:f>IF(OR($G43="",$H43="",$H43&lt;$G43),"",IF(AND(K$9&lt;=$H43,K$9+6&gt;=$G43),1,""))</x:f>
       </x:c>
-      <x:c r="L43" s="70" t="str">
+      <x:c r="L43" s="70" t="n">
         <x:f>IF(OR($G43="",$H43="",$H43&lt;$G43),"",IF(AND(L$9&lt;=$H43,L$9+6&gt;=$G43),1,""))</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M43" s="70" t="n">
         <x:f>IF(OR($G43="",$H43="",$H43&lt;$G43),"",IF(AND(M$9&lt;=$H43,M$9+6&gt;=$G43),1,""))</x:f>
@@ -5141,7 +5142,7 @@
     </x:row>
     <x:row r="50" ht="72" customHeight="1">
       <x:c r="B50" s="61" t="str">
-        <x:v>Fuentes: REVISION-Y-PLAN.md; BACKLOG.csv; METRICAS.csv; VALIDACION.md; Search Console y GA4 consultados el 21/09/2026. GSC 23/08–19/09 vs 26/07–22/08: 296 vs 192 clics, 14 mil vs 9,55 mil impresiones, CTR 2,1% vs 2,0%, posición 8,4 vs 8,5. Auditoría GSC: 3.187 indexadas / 326 no indexadas; sitemap correcto con 29 páginas descubiertas; HTTPS 31/0; 2 enlaces externos y 7.751 internos; 662 oportunidades Merchant; sin acciones manuales ni problemas de seguridad; sin datos CrUX. GA4 24/08–20/09: 143 usuarios, 512 eventos, 178 page_view y 18 click; generate_lead aún no aparece. Jev 21/09: embudo/CTA 64% (confianza 0,56); enlaces/rich results 39% y asociación GA4 32% como segundo orden (confianza 0,23); Merchant 6% y outreach 26% a favor. G07 pasa a P0/en curso; G17 a P1. Las fechas futuras son planificación y se revisan semanalmente. G02 25/09: 64/47.727 ofertas disponibles con observación ≤24 h antes del ciclo medido; 80 observaciones persistidas en 11 tiendas en run 36164068314; despacho automático verificado en runs 36165637147 y 36166218562. G02 sigue en observación; próxima revisión tras siete ciclos útiles medidos el 03/10. Fuente: VALIDACION.md y FRESCURA-TIENDAS-2026-09-25.csv. Actualización 27/09/2026: PLAN-ADSENSE-2026-09-27.md y BACKLOG.csv G18–G26. Fechas propuestas y dependientes de cuenta, contenido, privacidad y aprobación externa; anuncios no activos. Cuenta existente confirmada por Jonathan; país y método de cobro requieren comprobación. Fuente de políticas: https://support.google.com/adsense/answer/9724?hl=es. QVL y difusión conservan sus cortes históricos. Corte 27/09: G21 iniciado, consentimiento GA4 básico y política implementados; 19 pruebas y navegador local desktop/móvil verificados. Publicación, recepción del contacto y CMP de anuncios pendientes. G19 mantiene revisión y registro de derechos pendiente. No aprobado para AdSense.</x:v>
+        <x:v>Fuentes: REVISION-Y-PLAN.md; BACKLOG.csv; METRICAS.csv; VALIDACION.md; Search Console y GA4 consultados el 21/09/2026. GSC 23/08–19/09 vs 26/07–22/08: 296 vs 192 clics, 14 mil vs 9,55 mil impresiones, CTR 2,1% vs 2,0%, posición 8,4 vs 8,5. Auditoría GSC: 3.187 indexadas / 326 no indexadas; sitemap correcto con 29 páginas descubiertas; HTTPS 31/0; 2 enlaces externos y 7.751 internos; 662 oportunidades Merchant; sin acciones manuales ni problemas de seguridad; sin datos CrUX. GA4 24/08–20/09: 143 usuarios, 512 eventos, 178 page_view y 18 click; generate_lead aún no aparece. Jev 21/09: embudo/CTA 64% (confianza 0,56); enlaces/rich results 39% y asociación GA4 32% como segundo orden (confianza 0,23); Merchant 6% y outreach 26% a favor. G07 pasa a P0/en curso; G17 a P1. Las fechas futuras son planificación y se revisan semanalmente. G02 25/09: 64/47.727 ofertas disponibles con observación ≤24 h antes del ciclo medido; 80 observaciones persistidas en 11 tiendas en run 36164068314; despacho automático verificado en runs 36165637147 y 36166218562. G02 sigue en observación; próxima revisión tras siete ciclos útiles medidos el 03/10. Fuente: VALIDACION.md y FRESCURA-TIENDAS-2026-09-25.csv. Actualización 27/09/2026: PLAN-ADSENSE-2026-09-27.md y BACKLOG.csv G18–G26. Fechas propuestas y dependientes de cuenta, contenido, privacidad y aprobación externa; anuncios no activos. Cuenta existente confirmada por Jonathan; país y método de cobro requieren comprobación. Fuente de políticas: https://support.google.com/adsense/answer/9724?hl=es. QVL y difusión conservan sus cortes históricos. Corte 27/09: G21 iniciado, consentimiento GA4 básico y política implementados; 19 pruebas y navegador local desktop/móvil verificados. Publicación, recepción del contacto y CMP de anuncios pendientes. G19 mantiene revisión y registro de derechos pendiente. No aprobado para AdSense. Corte 27/09: G20 en revisión. Tres piezas con metodología y fuentes preparadas; 43 pruebas, lint y build. G21: 20 pruebas y flujo público de consentimiento desktop/móvil verificado después de corregir configuración servidor/navegador. Falta revisión humana, registro de derechos, recepción de contacto, perfil de pagos y CMP. Solicitud no enviada.</x:v>
       </x:c>
       <x:c r="C50" s="61"/>
       <x:c r="D50" s="61"/>

</xml_diff>

<commit_message>
docs(adsense): close ownership verification and inventory asset rights
</commit_message>
<xml_diff>
--- a/outputs/project-tracker-2026-09-27-adsense/Comparador-Hardware-Project-Tracker.xlsx
+++ b/outputs/project-tracker-2026-09-27-adsense/Comparador-Hardware-Project-Tracker.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Plan" sheetId="1" r:id="R38f1cadb5da44abf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Plan" sheetId="1" r:id="R789ef7d1579b4a40"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1247,7 +1247,7 @@
       <x:c r="N6" s="44"/>
       <x:c r="O6" s="45" t="n">
         <x:f>COUNTIF($E$10:$E$49,"Complete")</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="P6" s="46"/>
       <x:c r="Q6" s="46"/>
@@ -4701,34 +4701,34 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="E45" s="66" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="F45" s="66" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="G45" s="68" t="n">
-        <x:v>46300.5</x:v>
+        <x:v>46292.5</x:v>
       </x:c>
       <x:c r="H45" s="68" t="n">
-        <x:v>46303.5</x:v>
+        <x:v>46292.5</x:v>
       </x:c>
       <x:c r="I45" s="69" t="n">
         <x:f>IF(OR(G45="",H45="",H45&lt;G45),"",H45-G45+1)</x:f>
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J45"/>
       <x:c r="K45" s="70" t="str">
         <x:f>IF(OR($G45="",$H45="",$H45&lt;$G45),"",IF(AND(K$9&lt;=$H45,K$9+6&gt;=$G45),1,""))</x:f>
       </x:c>
-      <x:c r="L45" s="70" t="str">
+      <x:c r="L45" s="70" t="n">
         <x:f>IF(OR($G45="",$H45="",$H45&lt;$G45),"",IF(AND(L$9&lt;=$H45,L$9+6&gt;=$G45),1,""))</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M45" s="70" t="str">
         <x:f>IF(OR($G45="",$H45="",$H45&lt;$G45),"",IF(AND(M$9&lt;=$H45,M$9+6&gt;=$G45),1,""))</x:f>
       </x:c>
-      <x:c r="N45" s="70" t="n">
+      <x:c r="N45" s="70" t="str">
         <x:f>IF(OR($G45="",$H45="",$H45&lt;$G45),"",IF(AND(N$9&lt;=$H45,N$9+6&gt;=$G45),1,""))</x:f>
-        <x:v>1</x:v>
       </x:c>
       <x:c r="O45" s="70" t="str">
         <x:f>IF(OR($G45="",$H45="",$H45&lt;$G45),"",IF(AND(O$9&lt;=$H45,O$9+6&gt;=$G45),1,""))</x:f>
@@ -5142,7 +5142,7 @@
     </x:row>
     <x:row r="50" ht="72" customHeight="1">
       <x:c r="B50" s="61" t="str">
-        <x:v>Fuentes: REVISION-Y-PLAN.md; BACKLOG.csv; METRICAS.csv; VALIDACION.md; Search Console y GA4 consultados el 21/09/2026. GSC 23/08–19/09 vs 26/07–22/08: 296 vs 192 clics, 14 mil vs 9,55 mil impresiones, CTR 2,1% vs 2,0%, posición 8,4 vs 8,5. Auditoría GSC: 3.187 indexadas / 326 no indexadas; sitemap correcto con 29 páginas descubiertas; HTTPS 31/0; 2 enlaces externos y 7.751 internos; 662 oportunidades Merchant; sin acciones manuales ni problemas de seguridad; sin datos CrUX. GA4 24/08–20/09: 143 usuarios, 512 eventos, 178 page_view y 18 click; generate_lead aún no aparece. Jev 21/09: embudo/CTA 64% (confianza 0,56); enlaces/rich results 39% y asociación GA4 32% como segundo orden (confianza 0,23); Merchant 6% y outreach 26% a favor. G07 pasa a P0/en curso; G17 a P1. Las fechas futuras son planificación y se revisan semanalmente. G02 25/09: 64/47.727 ofertas disponibles con observación ≤24 h antes del ciclo medido; 80 observaciones persistidas en 11 tiendas en run 36164068314; despacho automático verificado en runs 36165637147 y 36166218562. G02 sigue en observación; próxima revisión tras siete ciclos útiles medidos el 03/10. Fuente: VALIDACION.md y FRESCURA-TIENDAS-2026-09-25.csv. Actualización 27/09/2026: PLAN-ADSENSE-2026-09-27.md y BACKLOG.csv G18–G26. Fechas propuestas y dependientes de cuenta, contenido, privacidad y aprobación externa; anuncios no activos. Cuenta existente confirmada por Jonathan; país y método de cobro requieren comprobación. Fuente de políticas: https://support.google.com/adsense/answer/9724?hl=es. QVL y difusión conservan sus cortes históricos. Corte 27/09: G21 iniciado, consentimiento GA4 básico y política implementados; 19 pruebas y navegador local desktop/móvil verificados. Publicación, recepción del contacto y CMP de anuncios pendientes. G19 mantiene revisión y registro de derechos pendiente. No aprobado para AdSense. Corte 27/09: G20 en revisión. Tres piezas con metodología y fuentes preparadas; 43 pruebas, lint y build. G21: 20 pruebas y flujo público de consentimiento desktop/móvil verificado después de corregir configuración servidor/navegador. Falta revisión humana, registro de derechos, recepción de contacto, perfil de pagos y CMP. Solicitud no enviada.</x:v>
+        <x:v>Fuentes: REVISION-Y-PLAN.md; BACKLOG.csv; METRICAS.csv; VALIDACION.md; Search Console y GA4 consultados el 21/09/2026. GSC 23/08–19/09 vs 26/07–22/08: 296 vs 192 clics, 14 mil vs 9,55 mil impresiones, CTR 2,1% vs 2,0%, posición 8,4 vs 8,5. Auditoría GSC: 3.187 indexadas / 326 no indexadas; sitemap correcto con 29 páginas descubiertas; HTTPS 31/0; 2 enlaces externos y 7.751 internos; 662 oportunidades Merchant; sin acciones manuales ni problemas de seguridad; sin datos CrUX. GA4 24/08–20/09: 143 usuarios, 512 eventos, 178 page_view y 18 click; generate_lead aún no aparece. Jev 21/09: embudo/CTA 64% (confianza 0,56); enlaces/rich results 39% y asociación GA4 32% como segundo orden (confianza 0,23); Merchant 6% y outreach 26% a favor. G07 pasa a P0/en curso; G17 a P1. Las fechas futuras son planificación y se revisan semanalmente. G02 25/09: 64/47.727 ofertas disponibles con observación ≤24 h antes del ciclo medido; 80 observaciones persistidas en 11 tiendas en run 36164068314; despacho automático verificado en runs 36165637147 y 36166218562. G02 sigue en observación; próxima revisión tras siete ciclos útiles medidos el 03/10. Fuente: VALIDACION.md y FRESCURA-TIENDAS-2026-09-25.csv. Actualización 27/09/2026: PLAN-ADSENSE-2026-09-27.md y BACKLOG.csv G18–G26. Fechas propuestas y dependientes de cuenta, contenido, privacidad y aprobación externa; anuncios no activos. Cuenta existente confirmada por Jonathan; país y método de cobro requieren comprobación. Fuente de políticas: https://support.google.com/adsense/answer/9724?hl=es. QVL y difusión conservan sus cortes históricos. Corte 27/09: G21 iniciado, consentimiento GA4 básico y política implementados; 19 pruebas y navegador local desktop/móvil verificados. Publicación, recepción del contacto y CMP de anuncios pendientes. G19 mantiene revisión y registro de derechos pendiente. No aprobado para AdSense. Corte 27/09: G20 en revisión. Tres piezas con metodología y fuentes preparadas; 43 pruebas, lint y build. G21: 20 pruebas y flujo público de consentimiento desktop/móvil verificado después de corregir configuración servidor/navegador. Falta revisión humana, registro de derechos, recepción de contacto, perfil de pagos y CMP. Solicitud no enviada. Corte 27/09: G22 cerrado. Dominio añadido en AdSense, metadato y ads.txt contrastados con cuenta y verificados públicamente en www/raíz; Google confirmó propiedad. Script de anuncios ausente, CSP sin nuevos orígenes. Revisión de sitio no solicitada. G18/G19/G20/G21/G23/G24 conservan dependencias abiertas.</x:v>
       </x:c>
       <x:c r="C50" s="61"/>
       <x:c r="D50" s="61"/>

</xml_diff>

<commit_message>
docs(adsense): record disabled pilot and tracker progress
</commit_message>
<xml_diff>
--- a/outputs/project-tracker-2026-09-27-adsense/Comparador-Hardware-Project-Tracker.xlsx
+++ b/outputs/project-tracker-2026-09-27-adsense/Comparador-Hardware-Project-Tracker.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Plan" sheetId="1" r:id="R789ef7d1579b4a40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Plan" sheetId="1" r:id="R91812e09cb9a4048"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1254,7 +1254,7 @@
       <x:c r="R6" s="47"/>
       <x:c r="S6" s="35" t="n">
         <x:f>COUNTIF($E$10:$E$49,"In Progress")</x:f>
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="T6" s="36"/>
       <x:c r="U6" s="36"/>
@@ -4790,30 +4790,32 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="E46" s="66" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="F46" s="66" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="G46" s="68" t="n">
-        <x:v>46300.5</x:v>
+        <x:v>46292.5</x:v>
       </x:c>
       <x:c r="H46" s="68" t="n">
         <x:v>46304.5</x:v>
       </x:c>
       <x:c r="I46" s="69" t="n">
         <x:f>IF(OR(G46="",H46="",H46&lt;G46),"",H46-G46+1)</x:f>
-        <x:v>5</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="J46"/>
       <x:c r="K46" s="70" t="str">
         <x:f>IF(OR($G46="",$H46="",$H46&lt;$G46),"",IF(AND(K$9&lt;=$H46,K$9+6&gt;=$G46),1,""))</x:f>
       </x:c>
-      <x:c r="L46" s="70" t="str">
+      <x:c r="L46" s="70" t="n">
         <x:f>IF(OR($G46="",$H46="",$H46&lt;$G46),"",IF(AND(L$9&lt;=$H46,L$9+6&gt;=$G46),1,""))</x:f>
-      </x:c>
-      <x:c r="M46" s="70" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M46" s="70" t="n">
         <x:f>IF(OR($G46="",$H46="",$H46&lt;$G46),"",IF(AND(M$9&lt;=$H46,M$9+6&gt;=$G46),1,""))</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N46" s="70" t="n">
         <x:f>IF(OR($G46="",$H46="",$H46&lt;$G46),"",IF(AND(N$9&lt;=$H46,N$9+6&gt;=$G46),1,""))</x:f>
@@ -5142,7 +5144,7 @@
     </x:row>
     <x:row r="50" ht="72" customHeight="1">
       <x:c r="B50" s="61" t="str">
-        <x:v>Fuentes: REVISION-Y-PLAN.md; BACKLOG.csv; METRICAS.csv; VALIDACION.md; Search Console y GA4 consultados el 21/09/2026. GSC 23/08–19/09 vs 26/07–22/08: 296 vs 192 clics, 14 mil vs 9,55 mil impresiones, CTR 2,1% vs 2,0%, posición 8,4 vs 8,5. Auditoría GSC: 3.187 indexadas / 326 no indexadas; sitemap correcto con 29 páginas descubiertas; HTTPS 31/0; 2 enlaces externos y 7.751 internos; 662 oportunidades Merchant; sin acciones manuales ni problemas de seguridad; sin datos CrUX. GA4 24/08–20/09: 143 usuarios, 512 eventos, 178 page_view y 18 click; generate_lead aún no aparece. Jev 21/09: embudo/CTA 64% (confianza 0,56); enlaces/rich results 39% y asociación GA4 32% como segundo orden (confianza 0,23); Merchant 6% y outreach 26% a favor. G07 pasa a P0/en curso; G17 a P1. Las fechas futuras son planificación y se revisan semanalmente. G02 25/09: 64/47.727 ofertas disponibles con observación ≤24 h antes del ciclo medido; 80 observaciones persistidas en 11 tiendas en run 36164068314; despacho automático verificado en runs 36165637147 y 36166218562. G02 sigue en observación; próxima revisión tras siete ciclos útiles medidos el 03/10. Fuente: VALIDACION.md y FRESCURA-TIENDAS-2026-09-25.csv. Actualización 27/09/2026: PLAN-ADSENSE-2026-09-27.md y BACKLOG.csv G18–G26. Fechas propuestas y dependientes de cuenta, contenido, privacidad y aprobación externa; anuncios no activos. Cuenta existente confirmada por Jonathan; país y método de cobro requieren comprobación. Fuente de políticas: https://support.google.com/adsense/answer/9724?hl=es. QVL y difusión conservan sus cortes históricos. Corte 27/09: G21 iniciado, consentimiento GA4 básico y política implementados; 19 pruebas y navegador local desktop/móvil verificados. Publicación, recepción del contacto y CMP de anuncios pendientes. G19 mantiene revisión y registro de derechos pendiente. No aprobado para AdSense. Corte 27/09: G20 en revisión. Tres piezas con metodología y fuentes preparadas; 43 pruebas, lint y build. G21: 20 pruebas y flujo público de consentimiento desktop/móvil verificado después de corregir configuración servidor/navegador. Falta revisión humana, registro de derechos, recepción de contacto, perfil de pagos y CMP. Solicitud no enviada. Corte 27/09: G22 cerrado. Dominio añadido en AdSense, metadato y ads.txt contrastados con cuenta y verificados públicamente en www/raíz; Google confirmó propiedad. Script de anuncios ausente, CSP sin nuevos orígenes. Revisión de sitio no solicitada. G18/G19/G20/G21/G23/G24 conservan dependencias abiertas.</x:v>
+        <x:v>Fuentes: REVISION-Y-PLAN.md; BACKLOG.csv; METRICAS.csv; VALIDACION.md; Search Console y GA4 consultados el 21/09/2026. GSC 23/08–19/09 vs 26/07–22/08: 296 vs 192 clics, 14 mil vs 9,55 mil impresiones, CTR 2,1% vs 2,0%, posición 8,4 vs 8,5. Auditoría GSC: 3.187 indexadas / 326 no indexadas; sitemap correcto con 29 páginas descubiertas; HTTPS 31/0; 2 enlaces externos y 7.751 internos; 662 oportunidades Merchant; sin acciones manuales ni problemas de seguridad; sin datos CrUX. GA4 24/08–20/09: 143 usuarios, 512 eventos, 178 page_view y 18 click; generate_lead aún no aparece. Jev 21/09: embudo/CTA 64% (confianza 0,56); enlaces/rich results 39% y asociación GA4 32% como segundo orden (confianza 0,23); Merchant 6% y outreach 26% a favor. G07 pasa a P0/en curso; G17 a P1. Las fechas futuras son planificación y se revisan semanalmente. G02 25/09: 64/47.727 ofertas disponibles con observación ≤24 h antes del ciclo medido; 80 observaciones persistidas en 11 tiendas en run 36164068314; despacho automático verificado en runs 36165637147 y 36166218562. G02 sigue en observación; próxima revisión tras siete ciclos útiles medidos el 03/10. Fuente: VALIDACION.md y FRESCURA-TIENDAS-2026-09-25.csv. Actualización 27/09/2026: PLAN-ADSENSE-2026-09-27.md y BACKLOG.csv G18–G26. Fechas propuestas y dependientes de cuenta, contenido, privacidad y aprobación externa; anuncios no activos. Cuenta existente confirmada por Jonathan; país y método de cobro requieren comprobación. Fuente de políticas: https://support.google.com/adsense/answer/9724?hl=es. QVL y difusión conservan sus cortes históricos. Corte 27/09: G21 iniciado, consentimiento GA4 básico y política implementados; 19 pruebas y navegador local desktop/móvil verificados. Publicación, recepción del contacto y CMP de anuncios pendientes. G19 mantiene revisión y registro de derechos pendiente. No aprobado para AdSense. Corte 27/09: G20 en revisión. Tres piezas con metodología y fuentes preparadas; 43 pruebas, lint y build. G21: 20 pruebas y flujo público de consentimiento desktop/móvil verificado después de corregir configuración servidor/navegador. Falta revisión humana, registro de derechos, recepción de contacto, perfil de pagos y CMP. Solicitud no enviada. Corte 27/09: G22 cerrado. Dominio añadido en AdSense, metadato y ads.txt contrastados con cuenta y verificados públicamente en www/raíz; Google confirmó propiedad. Script de anuncios ausente, CSP sin nuevos orígenes. Revisión de sitio no solicitada. G18/G19/G20/G21/G23/G24 conservan dependencias abiertas. Corte 27/09: G23 en revisión. Bloque real 300x250 creado; maqueta local en tres rutas, oculta en producción. Pruebas 320/390/1280 sin peticiones de anuncios. CMP y entrega real pendientes antes de activar.</x:v>
       </x:c>
       <x:c r="C50" s="61"/>
       <x:c r="D50" s="61"/>

</xml_diff>